<commit_message>
hiển thị tình trạng xác nhận đúc và cán
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC1_BBXNSL_PhoiTam.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC1_BBXNSL_PhoiTam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\BIEUMAU_SANXUAT\Source\dataproduct.BE\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CAFCFD-52B1-4ACE-8B8A-DDAA8AF49697}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE571B38-31BC-4748-8303-702417FADDFF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11805" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
   </bookViews>
@@ -25,18 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Mác thép</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Ghi chú</t>
   </si>
   <si>
     <t>STT</t>
-  </si>
-  <si>
-    <t>Sản phẩm</t>
   </si>
   <si>
     <t>Số phôi</t>
@@ -51,6 +45,9 @@
   </si>
   <si>
     <t xml:space="preserve">BIÊN BẢN XÁC NHẬN SẢN LƯỢNG PHÔI TẤM </t>
+  </si>
+  <si>
+    <t>Sản phẩm x Mác thép</t>
   </si>
 </sst>
 </file>
@@ -106,7 +103,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -138,16 +135,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -523,84 +536,76 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FE70C8B-98CB-4803-B542-3EE340B9292E}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="38.5703125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="35.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="33.5703125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="35.140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" style="2" customWidth="1"/>
-    <col min="9" max="10" width="9.140625" style="2"/>
-    <col min="11" max="11" width="13.140625" style="2" customWidth="1"/>
-    <col min="12" max="12" width="13.42578125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" style="2" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="2"/>
+    <col min="3" max="3" width="17.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="33.5703125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="35.140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" style="2" customWidth="1"/>
+    <col min="8" max="9" width="9.140625" style="2"/>
+    <col min="10" max="10" width="13.140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+    </row>
+    <row r="2" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+    </row>
+    <row r="4" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-    </row>
-    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-    </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-    </row>
-    <row r="4" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F4"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>